<commit_message>
feat: login/logout com usuario EstratOpera - todas as paginas protegidas
</commit_message>
<xml_diff>
--- a/Controle de Licenças Fortinet (estudo) 1.xlsx
+++ b/Controle de Licenças Fortinet (estudo) 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hitssbr-my.sharepoint.com/personal/carlos_costato_globalhitss_com_br/Documents/Documents/Calculadora/sistema_py/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D475751-712C-4EFA-9145-51B953F841D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{5D475751-712C-4EFA-9145-51B953F841D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE430E0F-B903-47E6-BC26-A52412125EAB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AF911547-A90A-4949-9F9B-1DCF6CA65B27}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{AF911547-A90A-4949-9F9B-1DCF6CA65B27}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="7" r:id="rId1"/>
@@ -6878,7 +6878,7 @@
   <dimension ref="A1:U82"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.21875" customWidth="1"/>
     <col min="2" max="2" width="20.88671875" customWidth="1"/>
     <col min="3" max="5" width="17.5546875" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" customWidth="1"/>

</xml_diff>